<commit_message>
Actualizar datos de Excel a JSON y añadir nuevas piezas M-073 y M-074
</commit_message>
<xml_diff>
--- a/Coleccion de minerales.xlsx
+++ b/Coleccion de minerales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Colección Minerales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDC0287-D640-4AA6-A656-EA82535B2BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F91A32-0DD6-4942-8E35-61D0623E7914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1353" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="584">
   <si>
     <t>Mineral</t>
   </si>
@@ -1880,6 +1880,35 @@
   </si>
   <si>
     <t>59x30x44</t>
+  </si>
+  <si>
+    <t>M-073</t>
+  </si>
+  <si>
+    <t>M-074</t>
+  </si>
+  <si>
+    <t>Taouz, Er Rachidia Province, Drâa-Tafilalet Region</t>
+  </si>
+  <si>
+    <t>Mibladen mining district, Midelt Province, Drâa-Tafilalet Region</t>
+  </si>
+  <si>
+    <t>Vítreo-Adamantino</t>
+  </si>
+  <si>
+    <t>95x30x35</t>
+  </si>
+  <si>
+    <t>80x50x45</t>
+  </si>
+  <si>
+    <t>Agregado estalactítico de goethita de color gris negruzco, con crecimiento fibroso y radiado, parcialmente recubierto por numerosos agregados y cristales blancos de calcita. Destaca por el fuerte contraste cromático y por su característica morfología vertical y escultórica.</t>
+  </si>
+  <si>
+    <t>Ejemplar de vanadinita de intenso color rojo anaranjado a rojo ladrillo, formando una profusa cubierta de cristales sobre una matriz de barita blanca a crema.
+Los cristales de vanadinita presentan hábito predominantemente prismático hexagonal corto y tabular, con numerosas terminaciones bien desarrolladas. Destaca especialmente el elevado número de individuos cristalinos que recubren prácticamente toda la superficie expuesta, creando una drusa densa y tridimensional.
+Entre los cristales se observan áreas de barita blanca, laminar y parcialmente cristalizada, que proporcionan un contraste cromático muy marcado.</t>
   </si>
 </sst>
 </file>
@@ -2333,7 +2362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z73"/>
+  <dimension ref="A1:Z75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -7378,6 +7407,139 @@
         <v>12</v>
       </c>
     </row>
+    <row r="74" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B74" t="s">
+        <v>180</v>
+      </c>
+      <c r="C74" t="s">
+        <v>374</v>
+      </c>
+      <c r="D74" t="s">
+        <v>40</v>
+      </c>
+      <c r="E74" t="s">
+        <v>440</v>
+      </c>
+      <c r="F74" t="s">
+        <v>336</v>
+      </c>
+      <c r="G74" t="s">
+        <v>343</v>
+      </c>
+      <c r="H74" t="s">
+        <v>430</v>
+      </c>
+      <c r="I74" t="s">
+        <v>386</v>
+      </c>
+      <c r="J74" t="s">
+        <v>305</v>
+      </c>
+      <c r="K74" t="s">
+        <v>332</v>
+      </c>
+      <c r="L74" t="s">
+        <v>296</v>
+      </c>
+      <c r="M74" t="s">
+        <v>580</v>
+      </c>
+      <c r="O74">
+        <v>63</v>
+      </c>
+      <c r="P74" t="s">
+        <v>577</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>18</v>
+      </c>
+      <c r="R74" t="s">
+        <v>300</v>
+      </c>
+      <c r="S74" t="s">
+        <v>373</v>
+      </c>
+      <c r="T74" s="6">
+        <v>46295</v>
+      </c>
+      <c r="U74">
+        <v>30</v>
+      </c>
+      <c r="V74" t="s">
+        <v>582</v>
+      </c>
+      <c r="W74" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="75" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="B75" t="s">
+        <v>57</v>
+      </c>
+      <c r="C75" t="s">
+        <v>374</v>
+      </c>
+      <c r="D75" t="s">
+        <v>137</v>
+      </c>
+      <c r="E75" t="s">
+        <v>381</v>
+      </c>
+      <c r="F75" t="s">
+        <v>363</v>
+      </c>
+      <c r="G75" t="s">
+        <v>335</v>
+      </c>
+      <c r="H75" t="s">
+        <v>315</v>
+      </c>
+      <c r="I75" t="s">
+        <v>307</v>
+      </c>
+      <c r="J75" t="s">
+        <v>579</v>
+      </c>
+      <c r="L75" t="s">
+        <v>296</v>
+      </c>
+      <c r="M75" t="s">
+        <v>581</v>
+      </c>
+      <c r="O75">
+        <v>215</v>
+      </c>
+      <c r="P75" t="s">
+        <v>578</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>18</v>
+      </c>
+      <c r="R75" t="s">
+        <v>300</v>
+      </c>
+      <c r="S75" t="s">
+        <v>373</v>
+      </c>
+      <c r="T75" s="6">
+        <v>46295</v>
+      </c>
+      <c r="U75">
+        <v>60</v>
+      </c>
+      <c r="V75" s="5" t="s">
+        <v>583</v>
+      </c>
+      <c r="W75" t="s">
+        <v>458</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>